<commit_message>
Add/Update Positions.xlsx via API
</commit_message>
<xml_diff>
--- a/BinancePTF/Positions.xlsx
+++ b/BinancePTF/Positions.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH860"/>
+  <dimension ref="A1:AH862"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -66655,6 +66655,130 @@
       </c>
       <c r="AH860" t="inlineStr"/>
     </row>
+    <row r="861">
+      <c r="A861" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B861" t="n">
+        <v>0.629026595</v>
+      </c>
+      <c r="C861" t="n">
+        <v>0.09801159550000001</v>
+      </c>
+      <c r="D861" t="inlineStr"/>
+      <c r="E861" t="inlineStr"/>
+      <c r="F861" t="inlineStr"/>
+      <c r="G861" t="inlineStr"/>
+      <c r="H861" t="inlineStr"/>
+      <c r="I861" t="n">
+        <v>0.05379677099999999</v>
+      </c>
+      <c r="J861" t="inlineStr"/>
+      <c r="K861" t="n">
+        <v>1559.126557421089</v>
+      </c>
+      <c r="L861" t="inlineStr"/>
+      <c r="M861" t="inlineStr"/>
+      <c r="N861" t="inlineStr"/>
+      <c r="O861" t="n">
+        <v>0.009360439</v>
+      </c>
+      <c r="P861" t="inlineStr"/>
+      <c r="Q861" t="n">
+        <v>1.0488e-06</v>
+      </c>
+      <c r="R861" t="inlineStr"/>
+      <c r="S861" t="inlineStr"/>
+      <c r="T861" t="inlineStr"/>
+      <c r="U861" t="inlineStr"/>
+      <c r="V861" t="inlineStr"/>
+      <c r="W861" t="inlineStr"/>
+      <c r="X861" t="inlineStr"/>
+      <c r="Y861" t="inlineStr"/>
+      <c r="Z861" t="inlineStr"/>
+      <c r="AA861" t="n">
+        <v>0.8384278614544</v>
+      </c>
+      <c r="AB861" t="n">
+        <v>242.925405408</v>
+      </c>
+      <c r="AC861" t="n">
+        <v>8.999358638272801</v>
+      </c>
+      <c r="AD861" t="n">
+        <v>0.153143965</v>
+      </c>
+      <c r="AE861" t="n">
+        <v>1812.861954809116</v>
+      </c>
+      <c r="AF861" t="inlineStr"/>
+      <c r="AG861" t="n">
+        <v>0.028865066</v>
+      </c>
+      <c r="AH861" t="inlineStr"/>
+    </row>
+    <row r="862">
+      <c r="A862" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B862" t="n">
+        <v>0.6293164</v>
+      </c>
+      <c r="C862" t="n">
+        <v>0.09773242750000001</v>
+      </c>
+      <c r="D862" t="inlineStr"/>
+      <c r="E862" t="inlineStr"/>
+      <c r="F862" t="inlineStr"/>
+      <c r="G862" t="inlineStr"/>
+      <c r="H862" t="inlineStr"/>
+      <c r="I862" t="n">
+        <v>0.05405376899999999</v>
+      </c>
+      <c r="J862" t="inlineStr"/>
+      <c r="K862" t="n">
+        <v>1554.929088376282</v>
+      </c>
+      <c r="L862" t="inlineStr"/>
+      <c r="M862" t="inlineStr"/>
+      <c r="N862" t="inlineStr"/>
+      <c r="O862" t="n">
+        <v>0.009424689999999999</v>
+      </c>
+      <c r="P862" t="inlineStr"/>
+      <c r="Q862" t="n">
+        <v>1.0464e-06</v>
+      </c>
+      <c r="R862" t="inlineStr"/>
+      <c r="S862" t="inlineStr"/>
+      <c r="T862" t="inlineStr"/>
+      <c r="U862" t="inlineStr"/>
+      <c r="V862" t="inlineStr"/>
+      <c r="W862" t="inlineStr"/>
+      <c r="X862" t="inlineStr"/>
+      <c r="Y862" t="inlineStr"/>
+      <c r="Z862" t="inlineStr"/>
+      <c r="AA862" t="n">
+        <v>0.8384530110207999</v>
+      </c>
+      <c r="AB862" t="n">
+        <v>233.26787441</v>
+      </c>
+      <c r="AC862" t="n">
+        <v>8.8316687257584</v>
+      </c>
+      <c r="AD862" t="n">
+        <v>0.15145806</v>
+      </c>
+      <c r="AE862" t="n">
+        <v>1798.837418971961</v>
+      </c>
+      <c r="AF862" t="inlineStr"/>
+      <c r="AG862" t="n">
+        <v>0.028348056</v>
+      </c>
+      <c r="AH862" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>